<commit_message>
Add highligh engineer and overall shifts excel generator
</commit_message>
<xml_diff>
--- a/data/Overall_Shifts_1404_2.xlsx
+++ b/data/Overall_Shifts_1404_2.xlsx
@@ -1336,7 +1336,11 @@
           <t>نصیری</t>
         </is>
       </c>
-      <c r="R24" s="7" t="n"/>
+      <c r="R24" s="7" t="inlineStr">
+        <is>
+          <t>حکم آبادی</t>
+        </is>
+      </c>
       <c r="S24" s="7" t="inlineStr">
         <is>
           <t>احسان پور</t>
@@ -1356,12 +1360,12 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>شرفی</t>
+          <t>عنایت فرد</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>نصیری</t>
+          <t>عنایت فرد</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -1371,7 +1375,7 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>رودی</t>
+          <t>علیپور</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
@@ -1491,11 +1495,7 @@
           <t>23 - سه‌شنبه</t>
         </is>
       </c>
-      <c r="Q26" s="7" t="inlineStr">
-        <is>
-          <t>نصیری</t>
-        </is>
-      </c>
+      <c r="Q26" s="7" t="n"/>
       <c r="R26" s="7" t="inlineStr">
         <is>
           <t>احسان پور</t>
@@ -1545,27 +1545,27 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
+          <t>رودی</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>24 - چهارشنبه</t>
+        </is>
+      </c>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
+          <t>علیپور</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="inlineStr">
+        <is>
           <t>شرفی</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr">
-        <is>
-          <t>24 - چهارشنبه</t>
-        </is>
-      </c>
-      <c r="L27" s="7" t="inlineStr">
-        <is>
-          <t>علیپور</t>
-        </is>
-      </c>
-      <c r="M27" s="7" t="inlineStr">
-        <is>
-          <t>شرفی</t>
-        </is>
-      </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>رودی</t>
+          <t>هاشمی</t>
         </is>
       </c>
       <c r="P27" s="3" t="inlineStr">
@@ -1603,47 +1603,47 @@
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
+          <t>بشک</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>25 - پنجشنبه</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>نظربیگی</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>فقیهی</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>رودی</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>25 - پنجشنبه</t>
+        </is>
+      </c>
+      <c r="L28" s="8" t="inlineStr">
+        <is>
           <t>شرفی</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>25 - پنجشنبه</t>
-        </is>
-      </c>
-      <c r="G28" s="8" t="inlineStr">
+      <c r="M28" s="8" t="inlineStr">
         <is>
           <t>علیپور</t>
         </is>
       </c>
-      <c r="H28" s="8" t="inlineStr">
-        <is>
-          <t>فقیهی</t>
-        </is>
-      </c>
-      <c r="I28" s="8" t="inlineStr">
-        <is>
-          <t>رودی</t>
-        </is>
-      </c>
-      <c r="K28" s="5" t="inlineStr">
-        <is>
-          <t>25 - پنجشنبه</t>
-        </is>
-      </c>
-      <c r="L28" s="8" t="inlineStr">
-        <is>
-          <t>هاشمی</t>
-        </is>
-      </c>
-      <c r="M28" s="8" t="inlineStr">
-        <is>
-          <t>شرفی</t>
-        </is>
-      </c>
       <c r="N28" s="8" t="inlineStr">
         <is>
-          <t>هاشمی</t>
+          <t>حکم آبادی</t>
         </is>
       </c>
       <c r="P28" s="5" t="inlineStr">
@@ -1676,27 +1676,27 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
+          <t>بشک</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>بشک</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>26 - جمعه</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>هاشمی</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
           <t>نوبخت</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>بشک</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>26 - جمعه</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>هاشمی</t>
-        </is>
-      </c>
-      <c r="H29" s="8" t="inlineStr">
-        <is>
-          <t>بشک</t>
         </is>
       </c>
       <c r="I29" s="8" t="inlineStr">
@@ -1750,47 +1750,47 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
+          <t>نظربیگی</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>نصیری</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>27 - شنبه</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>نظربیگی</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>شرفی</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>عنایت فرد</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>27 - شنبه</t>
+        </is>
+      </c>
+      <c r="L30" s="7" t="inlineStr">
+        <is>
+          <t>علیرضائی</t>
+        </is>
+      </c>
+      <c r="M30" s="7" t="inlineStr">
+        <is>
           <t>علیپور</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>نصیری</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>27 - شنبه</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
-        <is>
-          <t>نظربیگی</t>
-        </is>
-      </c>
-      <c r="H30" s="7" t="inlineStr">
-        <is>
-          <t>شرفی</t>
-        </is>
-      </c>
-      <c r="I30" s="7" t="inlineStr">
-        <is>
-          <t>دودانگه</t>
-        </is>
-      </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t>27 - شنبه</t>
-        </is>
-      </c>
-      <c r="L30" s="7" t="inlineStr">
-        <is>
-          <t>علیرضائی</t>
-        </is>
-      </c>
-      <c r="M30" s="7" t="inlineStr">
-        <is>
-          <t>نظربیگی</t>
         </is>
       </c>
       <c r="N30" s="7" t="inlineStr">
@@ -1828,47 +1828,47 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
+          <t>نظربیگی</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>بشک</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>28 - یکشنبه</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
           <t>علیپور</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="H31" s="7" t="inlineStr">
         <is>
           <t>بشک</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>عنایت فرد</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>28 - یکشنبه</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="L31" s="7" t="inlineStr">
+        <is>
+          <t>علیرضائی</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="inlineStr">
         <is>
           <t>علیپور</t>
-        </is>
-      </c>
-      <c r="H31" s="7" t="inlineStr">
-        <is>
-          <t>بشک</t>
-        </is>
-      </c>
-      <c r="I31" s="7" t="inlineStr">
-        <is>
-          <t>عنایت فرد</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t>28 - یکشنبه</t>
-        </is>
-      </c>
-      <c r="L31" s="7" t="inlineStr">
-        <is>
-          <t>علیرضائی</t>
-        </is>
-      </c>
-      <c r="M31" s="7" t="inlineStr">
-        <is>
-          <t>نظربیگی</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr">
@@ -2079,47 +2079,47 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
+          <t>رودی</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>31 - چهارشنبه</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
           <t>شریفی</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>علیپور</t>
+        </is>
+      </c>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>عنایت فرد</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
         <is>
           <t>31 - چهارشنبه</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="L34" s="7" t="inlineStr">
+        <is>
+          <t>علیرضائی</t>
+        </is>
+      </c>
+      <c r="M34" s="7" t="inlineStr">
+        <is>
+          <t>رودی</t>
+        </is>
+      </c>
+      <c r="N34" s="7" t="inlineStr">
         <is>
           <t>شریفی</t>
-        </is>
-      </c>
-      <c r="H34" s="7" t="inlineStr">
-        <is>
-          <t>علیپور</t>
-        </is>
-      </c>
-      <c r="I34" s="7" t="inlineStr">
-        <is>
-          <t>عنایت فرد</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr">
-        <is>
-          <t>31 - چهارشنبه</t>
-        </is>
-      </c>
-      <c r="L34" s="7" t="inlineStr">
-        <is>
-          <t>علیرضائی</t>
-        </is>
-      </c>
-      <c r="M34" s="7" t="inlineStr">
-        <is>
-          <t>رودی</t>
-        </is>
-      </c>
-      <c r="N34" s="7" t="inlineStr">
-        <is>
-          <t>هاشمی</t>
         </is>
       </c>
       <c r="P34" s="3" t="inlineStr">

</xml_diff>